<commit_message>
fix: /preferencias avisa qué palabras no guardó cuando pasan de 15 (BUG-32)
</commit_message>
<xml_diff>
--- a/docs/testing/casos-de-prueba-proyecto1.xlsx
+++ b/docs/testing/casos-de-prueba-proyecto1.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="240">
   <si>
     <t xml:space="preserve">Casos de prueba E2E del Proyecto 1 (job-search-agent)</t>
   </si>
@@ -843,6 +843,9 @@
   </si>
   <si>
     <t xml:space="preserve">Después de reiniciar, el bot no recibe mensajes y start-local.sh dice "Listo"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corregido y probado (2026-10-10)</t>
   </si>
   <si>
     <t xml:space="preserve">El BUG-36 apareció durante el caso E2E-23. El detalle completo de cada bug está en docs/bitacora-bugs.md.</t>
@@ -2839,7 +2842,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
         <v>236</v>
       </c>
@@ -2856,7 +2859,7 @@
         <v>171</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>231</v>
@@ -2864,7 +2867,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: /vacante muestra el número de la vacante guardada o repetida (BUG-33)
</commit_message>
<xml_diff>
--- a/docs/testing/casos-de-prueba-proyecto1.xlsx
+++ b/docs/testing/casos-de-prueba-proyecto1.xlsx
@@ -419,8 +419,8 @@
 - La respuesta muestra su número para usar /detalle.</t>
   </si>
   <si>
-    <t xml:space="preserve">- "Guardé la vacante (LinkedIn)" con el link limpio (jobs/view/4477446145).
-- La respuesta no muestra el número. En /nuevas aparece como #367.</t>
+    <t xml:space="preserve">- Primera ejecución (8 oct): "Guardé la vacante (LinkedIn)" con el link limpio (jobs/view/4477446145), pero sin número. En /nuevas aparece como #367 (BUG-33).
+- Re-test (10 oct, después de corregir BUG-33): "Guardé la vacante #400 (LinkedIn)" con /detalle 400, /guardar 400 y /descartar 400.</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-33</t>
@@ -445,7 +445,8 @@
   <si>
     <t xml:space="preserve">- "Esa vacante ya la tenías guardada (LinkedIn)" con el título de BairesDev.
 - En /nuevas no apareció otra copia.
-- La respuesta tampoco muestra el número (BUG-33).</t>
+- La respuesta tampoco muestra el número (BUG-33).
+- Re-test (10 oct): "Esa vacante ya la tenías guardada (#400, LinkedIn)", el mismo número de cuando se guardó. En /nuevas aparece una sola vez.</t>
   </si>
   <si>
     <t xml:space="preserve">EXP-02</t>
@@ -592,8 +593,9 @@
     <t xml:space="preserve">- El bot guarda las palabras nuevas, o avisa si alguna no se pudo guardar.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Responde "Listo, actualicé tu búsqueda", pero guarda solo 15. "tester" se descarta sin aviso.
-- Además, /preferencias con una sola palabra reemplaza toda la lista sin advertir.</t>
+    <t xml:space="preserve">- Primera ejecución (8 oct): responde "Listo, actualicé tu búsqueda", pero guarda solo 15. "tester" se descarta sin aviso (BUG-32).
+- Re-test (10 oct, después de corregir BUG-32): guarda 15 y avisa "No guardé: tester". Con las 15 de siempre responde "Listo" sin aviso.
+- Queda como observación que /preferencias con una sola palabra reemplaza toda la lista sin advertir.</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-32</t>
@@ -821,7 +823,7 @@
     <t xml:space="preserve">Media</t>
   </si>
   <si>
-    <t xml:space="preserve">Abierto</t>
+    <t xml:space="preserve">Corregido y probado (2026-10-10)</t>
   </si>
   <si>
     <t xml:space="preserve">Ver en la bitácora</t>
@@ -836,6 +838,9 @@
     <t xml:space="preserve">Alta</t>
   </si>
   <si>
+    <t xml:space="preserve">Corregido, falta re-test</t>
+  </si>
+  <si>
     <t xml:space="preserve">El filtro de ubicación deja pasar México escrito "MEX" o "CMX"</t>
   </si>
   <si>
@@ -843,9 +848,6 @@
   </si>
   <si>
     <t xml:space="preserve">Después de reiniciar, el bot no recibe mensajes y start-local.sh dice "Listo"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corregido y probado (2026-10-10)</t>
   </si>
   <si>
     <t xml:space="preserve">El BUG-36 apareció durante el caso E2E-23. El detalle completo de cada bug está en docs/bitacora-bugs.md.</t>
@@ -1368,15 +1370,15 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">COUNTIF(Radar!G2:G100,"Passed")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">COUNTIF(Radar!G2:G100,"Failed")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">IF(B7=0,"-",C7/B7)</f>
-        <v>0.714285714285714</v>
+        <v>0.857142857142857</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1389,15 +1391,15 @@
       </c>
       <c r="C8" s="4" t="n">
         <f aca="false">COUNTIF('Consultas por Telegram'!G2:G100,"Passed")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="4" t="n">
         <f aca="false">COUNTIF('Consultas por Telegram'!G2:G100,"Failed")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">IF(B8=0,"-",C8/B8)</f>
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1473,15 +1475,15 @@
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">SUM(C5:C11)</f>
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">SUM(D5:D11)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">IF(B12=0,"-",C12/B12)</f>
-        <v>0.875</v>
+        <v>0.9375</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,7 +2004,7 @@
       </c>
       <c r="H3" s="10"/>
     </row>
-    <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>108</v>
       </c>
@@ -2022,13 +2024,13 @@
         <v>113</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>115</v>
       </c>
@@ -2263,7 +2265,7 @@
       </c>
       <c r="H4" s="10"/>
     </row>
-    <row r="5" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>158</v>
       </c>
@@ -2283,7 +2285,7 @@
         <v>163</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>164</v>
@@ -2750,7 +2752,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
         <v>164</v>
       </c>
@@ -2773,7 +2775,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
         <v>114</v>
       </c>
@@ -2796,7 +2798,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>177</v>
       </c>
@@ -2813,18 +2815,18 @@
         <v>171</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>139</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>229</v>
@@ -2836,7 +2838,7 @@
         <v>133</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>231</v>
@@ -2844,10 +2846,10 @@
     </row>
     <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>229</v>
@@ -2859,7 +2861,7 @@
         <v>171</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>231</v>

</xml_diff>

<commit_message>
docs: cierre del Proyecto 1 (re-tests de BUG-34 y BUG-35, 32/32 casos, datos de ayudantes anonimizados)
</commit_message>
<xml_diff>
--- a/docs/testing/casos-de-prueba-proyecto1.xlsx
+++ b/docs/testing/casos-de-prueba-proyecto1.xlsx
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Casos de prueba E2E del Proyecto 1 (job-search-agent)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ejecutados del 7 al 10 de octubre de 2026 por Andrea Rivera. Detalle y evidencias en docs/testing/plan-pruebas-e2e.md.</t>
+    <t xml:space="preserve">Ejecutados del 7 al 11 de octubre de 2026 por Andrea Rivera, incluidos los re-tests de los 5 defectos. Detalle y evidencias en docs/testing/plan-pruebas-e2e.md.</t>
   </si>
   <si>
     <t xml:space="preserve">Hoja</t>
@@ -501,7 +501,8 @@
     <t xml:space="preserve">- Ninguna vacante de otro país (por ejemplo México).</t>
   </si>
   <si>
-    <t xml:space="preserve">- Pasó con la muestra de las 14:33, pero a las 5:24 p. m. llegó un aviso con vacantes en "Huixquilucán, MEX" y "Polanco, CMX".</t>
+    <t xml:space="preserve">- Primera ejecución (8 y 9 oct): pasó con la muestra de las 14:33, pero a las 5:24 p. m. llegó un aviso con vacantes en "Huixquilucán, MEX" y "Polanco, CMX" (BUG-35).
+- Re-test (11 oct, prueba controlada con curl a /radar/email): 3 vacantes de QA en "Huixquilucán, MEX", "Polanco, CMX" y "Zapopan, Jalisco". Resultado: found 3, skipped 3, created 0.</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-35</t>
@@ -642,7 +643,9 @@
   <si>
     <t xml:space="preserve">- El resumen sí respeta la pausa: el del 10 oct corrió sin incluirme.
 - Pero llegaron avisos de Indeed y LinkedIn a las 9:47 p. m. y 10:28 p. m.
-- /reanudar responde "¡Bienvenida/o de vuelta! Tu radar está activo otra vez."</t>
+- /reanudar responde "¡Bienvenida/o de vuelta! Tu radar está activo otra vez."
+- Re-test (10 oct, después de corregir BUG-34): en pausa llegó una vacante nueva por correo; se guardó (created 1) pero avisar salió false y no llegó nada a Telegram.
+- Regresión (10 y 11 oct): al reanudar, los avisos de correo volvieron a llegar.</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-34</t>
@@ -838,7 +841,7 @@
     <t xml:space="preserve">Alta</t>
   </si>
   <si>
-    <t xml:space="preserve">Corregido, falta re-test</t>
+    <t xml:space="preserve">Corregido y probado (2026-10-11)</t>
   </si>
   <si>
     <t xml:space="preserve">El filtro de ubicación deja pasar México escrito "MEX" o "CMX"</t>
@@ -1370,15 +1373,15 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">COUNTIF(Radar!G2:G100,"Passed")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">COUNTIF(Radar!G2:G100,"Failed")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">IF(B7=0,"-",C7/B7)</f>
-        <v>0.857142857142857</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1391,15 +1394,15 @@
       </c>
       <c r="C8" s="4" t="n">
         <f aca="false">COUNTIF('Consultas por Telegram'!G2:G100,"Passed")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="4" t="n">
         <f aca="false">COUNTIF('Consultas por Telegram'!G2:G100,"Failed")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">IF(B8=0,"-",C8/B8)</f>
-        <v>0.833333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1475,15 +1478,15 @@
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">SUM(C5:C11)</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">SUM(D5:D11)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">IF(B12=0,"-",C12/B12)</f>
-        <v>0.9375</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2102,7 +2105,7 @@
       </c>
       <c r="H7" s="10"/>
     </row>
-    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>133</v>
       </c>
@@ -2122,7 +2125,7 @@
         <v>138</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>139</v>
@@ -2315,7 +2318,7 @@
       </c>
       <c r="H6" s="10"/>
     </row>
-    <row r="7" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
         <v>171</v>
       </c>
@@ -2335,7 +2338,7 @@
         <v>176</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>177</v>
@@ -2798,7 +2801,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>177</v>
       </c>
@@ -2821,7 +2824,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>139</v>
       </c>

</xml_diff>